<commit_message>
Cập nhật import user
</commit_message>
<xml_diff>
--- a/packages/sohoa-backend/assets/user-import-template.xlsx
+++ b/packages/sohoa-backend/assets/user-import-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CE328F3-F7BE-4802-B35C-5C1EE47665C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D36130EB-714A-4ACD-903A-694DCE9955E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Email</t>
   </si>
@@ -61,19 +61,31 @@
   </si>
   <si>
     <t/>
+  </si>
+  <si>
+    <t>Role</t>
+  </si>
+  <si>
+    <t>admin/editer/qc</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="3">
@@ -85,8 +97,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
+        <fgColor rgb="FF4472C4"/>
       </patternFill>
     </fill>
   </fills>
@@ -102,9 +113,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -444,8 +458,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.796875" customWidth="1"/>
     <col min="2" max="2" width="14.796875" customWidth="1"/>
@@ -453,9 +467,10 @@
     <col min="4" max="4" width="12.796875" customWidth="1"/>
     <col min="5" max="5" width="16.796875" customWidth="1"/>
     <col min="6" max="6" width="12.796875" customWidth="1"/>
+    <col min="7" max="7" width="14.796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -474,8 +489,11 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="G1" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="2" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -493,12 +511,15 @@
       </c>
       <c r="F2" t="s">
         <v>11</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A2:F2 B1:F1" numberStoredAsText="1"/>
+    <ignoredError sqref="A2:F2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update import excel & assign folder
</commit_message>
<xml_diff>
--- a/packages/sohoa-backend/assets/user-import-template.xlsx
+++ b/packages/sohoa-backend/assets/user-import-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Sohoa_BE\sohoa-be\packages\sohoa-backend\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F477AE09-4A36-4121-93CD-C0BA1C0523B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C3D28F8-44F9-45EA-B6A5-FD22FB64FAD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>Email</t>
   </si>
@@ -64,6 +64,15 @@
   </si>
   <si>
     <t>2011-02-21</t>
+  </si>
+  <si>
+    <t>Password</t>
+  </si>
+  <si>
+    <t>abcz1234</t>
+  </si>
+  <si>
+    <t>0912345678</t>
   </si>
 </sst>
 </file>
@@ -111,12 +120,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -456,62 +466,68 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.59765625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="19.796875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="10.796875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="14.3984375" style="2" customWidth="1"/>
-    <col min="5" max="5" width="15.296875" style="2" customWidth="1"/>
-    <col min="6" max="6" width="10.796875" style="2" customWidth="1"/>
-    <col min="7" max="7" width="11.69921875" style="2" customWidth="1"/>
-    <col min="8" max="16384" width="8.796875" style="2"/>
+    <col min="1" max="2" width="21.59765625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="19.796875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="10.796875" style="2" customWidth="1"/>
+    <col min="5" max="5" width="14.3984375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="16.8984375" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.5" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.69921875" style="2" customWidth="1"/>
+    <col min="9" max="16384" width="8.796875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="2">
-        <v>912345678</v>
-      </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>12</v>
       </c>
     </row>

</xml_diff>